<commit_message>
tambahan beberapa komponen sama penyesuaian logika
</commit_message>
<xml_diff>
--- a/rosa_summary.xlsx
+++ b/rosa_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH10"/>
+  <dimension ref="A1:AH18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -938,50 +938,30 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>2</v>
       </c>
       <c r="H10" t="n">
         <v>1</v>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
         <v>2</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>1</v>
       </c>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
         <v>2</v>
       </c>
-      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
         <v>2</v>
       </c>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
         <v>1</v>
       </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
       <c r="X10" t="n">
         <v>2</v>
       </c>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="n">
         <v>1</v>
       </c>
@@ -998,6 +978,298 @@
         <v>3</v>
       </c>
       <c r="AH10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2</v>
+      </c>
+      <c r="P11" t="n">
+        <v>2</v>
+      </c>
+      <c r="T11" t="n">
+        <v>2</v>
+      </c>
+      <c r="X11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="J12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>2</v>
+      </c>
+      <c r="X12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" t="n">
+        <v>2</v>
+      </c>
+      <c r="X13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2</v>
+      </c>
+      <c r="O14" t="n">
+        <v>2</v>
+      </c>
+      <c r="X14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="J15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O15" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>2</v>
+      </c>
+      <c r="U15" t="n">
+        <v>2</v>
+      </c>
+      <c r="X15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2</v>
+      </c>
+      <c r="O16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2</v>
+      </c>
+      <c r="X17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="n">
+        <v>2</v>
+      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH18" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>